<commit_message>
Initial commit: Project structure setup with backend and frontend
</commit_message>
<xml_diff>
--- a/PRD/测试业务使用数据.xlsx
+++ b/PRD/测试业务使用数据.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>年份</t>
   </si>
@@ -50,73 +50,10 @@
     <t>问卷调查</t>
   </si>
   <si>
-    <t>医院信息调研管理</t>
-  </si>
-  <si>
     <t>科室信息调研管理</t>
   </si>
   <si>
-    <t>商业信息调研</t>
-  </si>
-  <si>
-    <t>竞品调研管理</t>
-  </si>
-  <si>
-    <t>义诊管理</t>
-  </si>
-  <si>
-    <t>会议管理</t>
-  </si>
-  <si>
-    <t>跟台管理</t>
-  </si>
-  <si>
-    <t>随访管理</t>
-  </si>
-  <si>
-    <t>药品流向管理</t>
-  </si>
-  <si>
-    <t>库存信息收集管理</t>
-  </si>
-  <si>
-    <t>品种准入</t>
-  </si>
-  <si>
-    <t>药店调研</t>
-  </si>
-  <si>
-    <t>会议报告</t>
-  </si>
-  <si>
-    <t>医院协访</t>
-  </si>
-  <si>
-    <t>药店协访</t>
-  </si>
-  <si>
-    <t>工作组药事报告</t>
-  </si>
-  <si>
-    <t>工作组市场容量调研报告</t>
-  </si>
-  <si>
-    <t>工作组竞品分析调研报告</t>
-  </si>
-  <si>
-    <t>月度推广计划</t>
-  </si>
-  <si>
     <t>工作组问卷调研分析报告</t>
-  </si>
-  <si>
-    <t>流向分析报告</t>
-  </si>
-  <si>
-    <t>库存分析报告</t>
-  </si>
-  <si>
-    <t>工作组报告</t>
   </si>
   <si>
     <t>2025</t>
@@ -782,23 +719,20 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1335,268 +1269,90 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AD5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="12.2019230769231" customWidth="1"/>
     <col min="2" max="2" width="11.625" customWidth="1"/>
     <col min="3" max="3" width="42.8557692307692" customWidth="1"/>
     <col min="4" max="7" width="16.2403846153846" customWidth="1"/>
-    <col min="8" max="9" width="27.4711538461538" customWidth="1"/>
-    <col min="10" max="11" width="22.8557692307692" customWidth="1"/>
-    <col min="12" max="15" width="16.2403846153846" customWidth="1"/>
-    <col min="16" max="16" width="22.8557692307692" customWidth="1"/>
-    <col min="17" max="17" width="27.4711538461538" customWidth="1"/>
-    <col min="18" max="22" width="16.2403846153846" customWidth="1"/>
-    <col min="23" max="23" width="25.1634615384615" customWidth="1"/>
-    <col min="24" max="25" width="18.6923076923077" customWidth="1"/>
-    <col min="26" max="26" width="22.8557692307692" customWidth="1"/>
-    <col min="27" max="27" width="18.6923076923077" customWidth="1"/>
-    <col min="28" max="29" width="22.8557692307692" customWidth="1"/>
-    <col min="30" max="30" width="18.5480769230769" customWidth="1"/>
+    <col min="8" max="8" width="27.4711538461538" customWidth="1"/>
+    <col min="9" max="9" width="49.2019230769231" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="48.5" customHeight="1" spans="1:30">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="1" customFormat="1" ht="48.5" customHeight="1" spans="1:9">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+    </row>
+    <row r="2" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:9">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="Z1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="AD1" s="4" t="s">
-        <v>29</v>
+      <c r="D2" s="6">
+        <v>1573</v>
+      </c>
+      <c r="E2" s="6">
+        <v>102</v>
+      </c>
+      <c r="F2" s="6">
+        <v>1733</v>
+      </c>
+      <c r="G2" s="6">
+        <v>415</v>
+      </c>
+      <c r="H2" s="6">
+        <v>1</v>
+      </c>
+      <c r="I2" s="6">
+        <v>4</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="30.5" customHeight="1" spans="1:30">
-      <c r="A2" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="7">
-        <v>1573</v>
-      </c>
-      <c r="E2" s="7">
-        <v>102</v>
-      </c>
-      <c r="F2" s="7">
-        <v>1733</v>
-      </c>
-      <c r="G2" s="7">
-        <v>415</v>
-      </c>
-      <c r="H2" s="7">
-        <v>0</v>
-      </c>
-      <c r="I2" s="7">
-        <v>1</v>
-      </c>
-      <c r="J2" s="7">
-        <v>0</v>
-      </c>
-      <c r="K2" s="7">
-        <v>0</v>
-      </c>
-      <c r="L2" s="7">
-        <v>0</v>
-      </c>
-      <c r="M2" s="7">
-        <v>0</v>
-      </c>
-      <c r="N2" s="7">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7">
-        <v>0</v>
-      </c>
-      <c r="P2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="7">
-        <v>0</v>
-      </c>
-      <c r="R2" s="7">
-        <v>0</v>
-      </c>
-      <c r="S2" s="7">
-        <v>0</v>
-      </c>
-      <c r="T2" s="7">
-        <v>0</v>
-      </c>
-      <c r="U2" s="7">
-        <v>0</v>
-      </c>
-      <c r="V2" s="7">
-        <v>0</v>
-      </c>
-      <c r="W2" s="7">
-        <v>0</v>
-      </c>
-      <c r="X2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="7">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="7">
-        <v>4</v>
-      </c>
-      <c r="AB2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="7">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="7">
-        <v>0</v>
-      </c>
+    <row r="4" s="1" customFormat="1" ht="18" customHeight="1" spans="1:9">
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
     </row>
-    <row r="4" s="2" customFormat="1" ht="18" customHeight="1" spans="1:30">
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="8"/>
-      <c r="W4" s="8"/>
-      <c r="X4" s="8"/>
-      <c r="Y4" s="8"/>
-      <c r="Z4" s="8"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="8"/>
-      <c r="AC4" s="8"/>
-      <c r="AD4" s="8"/>
-    </row>
-    <row r="5" s="2" customFormat="1" ht="18" customHeight="1" spans="1:30">
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="8"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8"/>
-      <c r="Y5" s="8"/>
-      <c r="Z5" s="8"/>
-      <c r="AA5" s="8"/>
-      <c r="AB5" s="8"/>
-      <c r="AC5" s="8"/>
-      <c r="AD5" s="8"/>
+    <row r="5" s="1" customFormat="1" ht="18" customHeight="1" spans="1:9">
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>